<commit_message>
Restore item 72 (The Drift Table) in data/timeline.xlsx
Restores the workbook exactly as it was at 2be103f, before the test
deletion in 4e12390. That upload changed nothing else.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jBG4cogwN8F7f83jnq38g
</commit_message>
<xml_diff>
--- a/data/timeline.xlsx
+++ b/data/timeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\romis\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC29EA6-B6AE-45EC-9E99-74E8D8AB4DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D42100-E05C-4A01-B857-894301C1BFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="454">
   <si>
     <t>id</t>
   </si>
@@ -794,6 +794,18 @@
   </si>
   <si>
     <t>Touch / Pen Interaction / Mobile Computing</t>
+  </si>
+  <si>
+    <t>The Drift Table</t>
+  </si>
+  <si>
+    <t>שולחן סלון אלקטרוני המציג תצלומי אוויר הנעים באיטיות בהתאם לחלוקת המשקל על פניו. כאשר המשתמש מניח חפצים או נשען על אזור מסוים, התצוגה נעה בכיוון המתאים ומאפשרת לשוטט בנופים ללא יעד מוגדר. המכשיר תוכנן לעודד סקרנות, משחק והתבוננות בבית, ולא לביצוע משימה שימושית, ושימש למחקר על עיצוב טכנולוגיות המעודדות חקירה חופשית.</t>
+  </si>
+  <si>
+    <t>ויליאם גייבר הוא מעצב וחוקר אינטראקציה שהתעניין בחוויה האנושית מעבר ליעילות ולשימושיות. מחקריו עוסקים במשחק, סקרנות, עמימות ודרכים שבהן טכנולוגיה יכולה לקבל משמעות אישית בחיי היומיום.</t>
+  </si>
+  <si>
+    <t>Tangible Interaction / Ambient Interaction</t>
   </si>
   <si>
     <t>Reactable Live</t>
@@ -1571,8 +1583,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1A74C817-109F-4704-9B2F-538DE84653E7}" name="טבלה1" displayName="טבלה1" ref="A1:P150" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="A1:P150" xr:uid="{1A74C817-109F-4704-9B2F-538DE84653E7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1A74C817-109F-4704-9B2F-538DE84653E7}" name="טבלה1" displayName="טבלה1" ref="A1:P151" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="A1:P151" xr:uid="{1A74C817-109F-4704-9B2F-538DE84653E7}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{F164D471-F0AB-430B-A6FB-6338D8DB3E2B}" name="id" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{F5ED8843-E467-4E3B-864E-7412714707BF}" name="era" dataDxfId="14"/>
@@ -1880,7 +1892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P150"/>
+  <dimension ref="A1:P151"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -1901,7 +1913,7 @@
     <col min="16" max="16" width="14.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4324,15 +4336,15 @@
       <c r="O69" s="3"/>
       <c r="P69" s="3"/>
     </row>
-    <row r="70" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C70" s="3">
-        <v>2005</v>
+        <v>2004</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
@@ -4344,8 +4356,11 @@
       <c r="G70" s="2" t="s">
         <v>246</v>
       </c>
+      <c r="H70" s="2" t="s">
+        <v>247</v>
+      </c>
       <c r="K70" s="2" t="s">
-        <v>144</v>
+        <v>248</v>
       </c>
       <c r="L70" s="3" t="s">
         <v>145</v>
@@ -4359,7 +4374,7 @@
     </row>
     <row r="71" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>120</v>
@@ -4372,65 +4387,63 @@
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="I71" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>81</v>
+        <v>144</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>82</v>
+        <v>145</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>83</v>
+        <v>146</v>
       </c>
       <c r="N71" s="3"/>
       <c r="O71" s="3"/>
       <c r="P71" s="3"/>
     </row>
-    <row r="72" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C72" s="3">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>253</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="L72" s="3" t="s">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N72" s="3">
-        <v>124</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="N72" s="3"/>
       <c r="O72" s="3"/>
       <c r="P72" s="3"/>
     </row>
     <row r="73" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>120</v>
@@ -4443,67 +4456,62 @@
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>181</v>
+        <v>22</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>181</v>
+        <v>22</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="N73" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="N73" s="3">
+        <v>124</v>
+      </c>
       <c r="O73" s="3"/>
       <c r="P73" s="3"/>
     </row>
-    <row r="74" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C74" s="3">
-        <v>2007</v>
+        <v>2006</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="H74" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>244</v>
+        <v>181</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>57</v>
+        <v>181</v>
       </c>
       <c r="M74" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="N74" s="3">
-        <v>142</v>
-      </c>
-      <c r="O74" s="3">
-        <v>120</v>
-      </c>
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
       <c r="P74" s="3"/>
     </row>
-    <row r="75" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>120</v>
@@ -4516,91 +4524,102 @@
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>260</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>145</v>
+        <v>244</v>
       </c>
       <c r="L75" s="3" t="s">
-        <v>145</v>
+        <v>57</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>146</v>
+        <v>58</v>
       </c>
       <c r="N75" s="3">
-        <v>141</v>
-      </c>
-      <c r="O75" s="3"/>
+        <v>142</v>
+      </c>
+      <c r="O75" s="3">
+        <v>120</v>
+      </c>
       <c r="P75" s="3"/>
     </row>
     <row r="76" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C76" s="3">
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="L76" s="3" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N76" s="3"/>
+        <v>146</v>
+      </c>
+      <c r="N76" s="3">
+        <v>141</v>
+      </c>
       <c r="O76" s="3"/>
       <c r="P76" s="3"/>
     </row>
-    <row r="77" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C77" s="3">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="E77" s="3"/>
       <c r="F77" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="K77" s="2"/>
-      <c r="L77" s="3"/>
-      <c r="M77" s="3"/>
-      <c r="N77" s="3">
-        <v>83</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="M77" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N77" s="3"/>
       <c r="O77" s="3"/>
       <c r="P77" s="3"/>
     </row>
-    <row r="78" spans="1:16" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>120</v>
@@ -4613,10 +4632,10 @@
       </c>
       <c r="E78" s="3"/>
       <c r="F78" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K78" s="2"/>
       <c r="L78" s="3"/>
@@ -4627,9 +4646,9 @@
       <c r="O78" s="3"/>
       <c r="P78" s="3"/>
     </row>
-    <row r="79" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>120</v>
@@ -4638,31 +4657,27 @@
         <v>2009</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="K79" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L79" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="M79" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N79" s="3"/>
+        <v>268</v>
+      </c>
+      <c r="K79" s="2"/>
+      <c r="L79" s="3"/>
+      <c r="M79" s="3"/>
+      <c r="N79" s="3">
+        <v>83</v>
+      </c>
       <c r="O79" s="3"/>
       <c r="P79" s="3"/>
     </row>
-    <row r="80" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>120</v>
@@ -4675,16 +4690,13 @@
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="I80" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>270</v>
+        <v>114</v>
       </c>
       <c r="L80" s="3" t="s">
         <v>115</v>
@@ -4692,22 +4704,16 @@
       <c r="M80" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="N80" s="3">
-        <v>59</v>
-      </c>
-      <c r="O80" s="3">
-        <v>80</v>
-      </c>
-      <c r="P80" s="3">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+      <c r="N80" s="3"/>
+      <c r="O80" s="3"/>
+      <c r="P80" s="3"/>
+    </row>
+    <row r="81" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>271</v>
+        <v>120</v>
       </c>
       <c r="C81" s="3">
         <v>2009</v>
@@ -4717,16 +4723,16 @@
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="G81" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="G81" s="2" t="s">
+      <c r="I81" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="H81" s="2" t="s">
+      <c r="K81" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="K81" s="2" t="s">
-        <v>275</v>
       </c>
       <c r="L81" s="3" t="s">
         <v>115</v>
@@ -4734,19 +4740,25 @@
       <c r="M81" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="N81" s="3"/>
-      <c r="O81" s="3"/>
-      <c r="P81" s="3"/>
-    </row>
-    <row r="82" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+      <c r="N81" s="3">
+        <v>59</v>
+      </c>
+      <c r="O81" s="3">
+        <v>80</v>
+      </c>
+      <c r="P81" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C82" s="3">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
@@ -4758,60 +4770,63 @@
       <c r="G82" s="2" t="s">
         <v>277</v>
       </c>
+      <c r="H82" s="2" t="s">
+        <v>278</v>
+      </c>
       <c r="K82" s="2" t="s">
-        <v>22</v>
+        <v>279</v>
       </c>
       <c r="L82" s="3" t="s">
-        <v>22</v>
+        <v>115</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N82" s="3">
-        <v>125</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="N82" s="3"/>
       <c r="O82" s="3"/>
       <c r="P82" s="3"/>
     </row>
     <row r="83" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C83" s="3">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="K83" s="2" t="s">
-        <v>280</v>
+        <v>22</v>
       </c>
       <c r="L83" s="3" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="N83" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="N83" s="3">
+        <v>125</v>
+      </c>
       <c r="O83" s="3"/>
       <c r="P83" s="3"/>
     </row>
-    <row r="84" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C84" s="3">
         <v>2011</v>
@@ -4821,30 +4836,30 @@
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K84" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L84" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="N84" s="3"/>
       <c r="O84" s="3"/>
       <c r="P84" s="3"/>
     </row>
-    <row r="85" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C85" s="3">
         <v>2011</v>
@@ -4854,71 +4869,66 @@
       </c>
       <c r="E85" s="3"/>
       <c r="F85" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="H85" s="2" t="s">
         <v>286</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>140</v>
+        <v>287</v>
       </c>
       <c r="L85" s="3" t="s">
-        <v>141</v>
+        <v>46</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="N85" s="3"/>
       <c r="O85" s="3"/>
       <c r="P85" s="3"/>
     </row>
-    <row r="86" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C86" s="3">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="I86" s="2" t="s">
         <v>289</v>
       </c>
+      <c r="H86" s="2" t="s">
+        <v>290</v>
+      </c>
       <c r="K86" s="2" t="s">
-        <v>173</v>
+        <v>140</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>174</v>
+        <v>141</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="N86" s="3">
-        <v>135</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="N86" s="3"/>
       <c r="O86" s="3"/>
       <c r="P86" s="3"/>
     </row>
     <row r="87" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C87" s="3">
         <v>2013</v>
@@ -4928,33 +4938,35 @@
       </c>
       <c r="E87" s="3"/>
       <c r="F87" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="K87" s="2" t="s">
-        <v>275</v>
+        <v>173</v>
       </c>
       <c r="L87" s="3" t="s">
-        <v>115</v>
+        <v>174</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N87" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="N87" s="3">
+        <v>135</v>
+      </c>
       <c r="O87" s="3"/>
       <c r="P87" s="3"/>
     </row>
-    <row r="88" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C88" s="3">
         <v>2013</v>
@@ -4964,30 +4976,33 @@
       </c>
       <c r="E88" s="3"/>
       <c r="F88" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
+      </c>
+      <c r="I88" s="2" t="s">
+        <v>296</v>
       </c>
       <c r="K88" s="2" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>22</v>
+        <v>115</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="N88" s="3"/>
       <c r="O88" s="3"/>
       <c r="P88" s="3"/>
     </row>
-    <row r="89" spans="1:16" ht="114" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C89" s="3">
         <v>2013</v>
@@ -4997,100 +5012,100 @@
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="K89" s="2" t="s">
-        <v>145</v>
+        <v>299</v>
       </c>
       <c r="L89" s="3" t="s">
-        <v>145</v>
+        <v>22</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="N89" s="3">
-        <v>141</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="N89" s="3"/>
       <c r="O89" s="3"/>
       <c r="P89" s="3"/>
     </row>
     <row r="90" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C90" s="3">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="K90" s="2" t="s">
-        <v>283</v>
+        <v>145</v>
       </c>
       <c r="L90" s="3" t="s">
-        <v>46</v>
+        <v>145</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>23</v>
+        <v>146</v>
       </c>
       <c r="N90" s="3">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="O90" s="3"/>
       <c r="P90" s="3"/>
     </row>
-    <row r="91" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C91" s="3">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="K91" s="2" t="s">
-        <v>115</v>
+        <v>287</v>
       </c>
       <c r="L91" s="3" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N91" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="N91" s="3">
+        <v>143</v>
+      </c>
       <c r="O91" s="3"/>
       <c r="P91" s="3"/>
     </row>
-    <row r="92" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C92" s="3">
         <v>2015</v>
@@ -5100,30 +5115,30 @@
       </c>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="L92" s="3" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>77</v>
+        <v>116</v>
       </c>
       <c r="N92" s="3"/>
       <c r="O92" s="3"/>
       <c r="P92" s="3"/>
     </row>
-    <row r="93" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C93" s="3">
         <v>2015</v>
@@ -5133,10 +5148,10 @@
       </c>
       <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="K93" s="2" t="s">
         <v>76</v>
@@ -5147,18 +5162,16 @@
       <c r="M93" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="N93" s="3">
-        <v>105</v>
-      </c>
+      <c r="N93" s="3"/>
       <c r="O93" s="3"/>
       <c r="P93" s="3"/>
     </row>
-    <row r="94" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C94" s="3">
         <v>2015</v>
@@ -5168,36 +5181,35 @@
       </c>
       <c r="E94" s="3"/>
       <c r="F94" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="I94" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K94" s="2" t="s">
-        <v>309</v>
+        <v>76</v>
       </c>
       <c r="L94" s="3" t="s">
-        <v>309</v>
+        <v>76</v>
       </c>
       <c r="M94" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="N94" s="3"/>
+      <c r="N94" s="3">
+        <v>105</v>
+      </c>
       <c r="O94" s="3"/>
       <c r="P94" s="3"/>
     </row>
-    <row r="95" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C95" s="3">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>17</v>
@@ -5209,25 +5221,28 @@
       <c r="G95" s="2" t="s">
         <v>311</v>
       </c>
+      <c r="I95" s="2" t="s">
+        <v>312</v>
+      </c>
       <c r="K95" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L95" s="3" t="s">
-        <v>68</v>
+        <v>313</v>
       </c>
       <c r="M95" s="3" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="N95" s="3"/>
       <c r="O95" s="3"/>
       <c r="P95" s="3"/>
     </row>
-    <row r="96" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C96" s="3">
         <v>2016</v>
@@ -5237,16 +5252,13 @@
       </c>
       <c r="E96" s="3"/>
       <c r="F96" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="J96" s="2" t="s">
         <v>315</v>
       </c>
       <c r="K96" s="2" t="s">
-        <v>68</v>
+        <v>316</v>
       </c>
       <c r="L96" s="3" t="s">
         <v>68</v>
@@ -5258,12 +5270,12 @@
       <c r="O96" s="3"/>
       <c r="P96" s="3"/>
     </row>
-    <row r="97" spans="1:16" ht="114" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C97" s="3">
         <v>2016</v>
@@ -5273,16 +5285,19 @@
       </c>
       <c r="E97" s="3"/>
       <c r="F97" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>319</v>
       </c>
       <c r="K97" s="2" t="s">
-        <v>318</v>
+        <v>68</v>
       </c>
       <c r="L97" s="3" t="s">
-        <v>319</v>
+        <v>68</v>
       </c>
       <c r="M97" s="3" t="s">
         <v>62</v>
@@ -5291,15 +5306,15 @@
       <c r="O97" s="3"/>
       <c r="P97" s="3"/>
     </row>
-    <row r="98" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C98" s="3">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>17</v>
@@ -5315,10 +5330,10 @@
         <v>322</v>
       </c>
       <c r="L98" s="3" t="s">
-        <v>115</v>
+        <v>323</v>
       </c>
       <c r="M98" s="3" t="s">
-        <v>116</v>
+        <v>62</v>
       </c>
       <c r="N98" s="3"/>
       <c r="O98" s="3"/>
@@ -5326,32 +5341,32 @@
     </row>
     <row r="99" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C99" s="3">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E99" s="3"/>
       <c r="F99" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>145</v>
+        <v>326</v>
       </c>
       <c r="L99" s="3" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="M99" s="3" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="N99" s="3"/>
       <c r="O99" s="3"/>
@@ -5359,53 +5374,46 @@
     </row>
     <row r="100" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C100" s="3">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E100" s="3"/>
       <c r="F100" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="H100" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K100" s="2" t="s">
-        <v>328</v>
+        <v>145</v>
       </c>
       <c r="L100" s="3" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="M100" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N100" s="3">
-        <v>26</v>
-      </c>
-      <c r="O100" s="3">
-        <v>128</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="N100" s="3"/>
+      <c r="O100" s="3"/>
       <c r="P100" s="3"/>
     </row>
-    <row r="101" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C101" s="3">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>17</v>
@@ -5417,60 +5425,67 @@
       <c r="G101" s="2" t="s">
         <v>330</v>
       </c>
+      <c r="H101" s="2" t="s">
+        <v>331</v>
+      </c>
       <c r="K101" s="2" t="s">
-        <v>76</v>
+        <v>332</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="M101" s="3" t="s">
-        <v>77</v>
+        <v>116</v>
       </c>
       <c r="N101" s="3">
-        <v>96</v>
-      </c>
-      <c r="O101" s="3"/>
+        <v>26</v>
+      </c>
+      <c r="O101" s="3">
+        <v>128</v>
+      </c>
       <c r="P101" s="3"/>
     </row>
-    <row r="102" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C102" s="3">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="K102" s="2" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="L102" s="3" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="M102" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N102" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="N102" s="3">
+        <v>96</v>
+      </c>
       <c r="O102" s="3"/>
       <c r="P102" s="3"/>
     </row>
-    <row r="103" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C103" s="3">
         <v>2021</v>
@@ -5480,19 +5495,19 @@
       </c>
       <c r="E103" s="3"/>
       <c r="F103" s="3" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="K103" s="2" t="s">
-        <v>173</v>
+        <v>21</v>
       </c>
       <c r="L103" s="3" t="s">
-        <v>174</v>
+        <v>22</v>
       </c>
       <c r="M103" s="3" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="N103" s="3"/>
       <c r="O103" s="3"/>
@@ -5500,48 +5515,43 @@
     </row>
     <row r="104" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>335</v>
+        <v>275</v>
       </c>
       <c r="C104" s="3">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E104" s="3"/>
       <c r="F104" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="I104" s="2" t="s">
         <v>338</v>
       </c>
       <c r="K104" s="2" t="s">
-        <v>126</v>
+        <v>173</v>
       </c>
       <c r="L104" s="3" t="s">
-        <v>126</v>
+        <v>174</v>
       </c>
       <c r="M104" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="N104" s="3">
-        <v>138</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="N104" s="3"/>
       <c r="O104" s="3"/>
       <c r="P104" s="3"/>
     </row>
-    <row r="105" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C105" s="3">
         <v>2022</v>
@@ -5551,19 +5561,16 @@
       </c>
       <c r="E105" s="3"/>
       <c r="F105" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="H105" s="2" t="s">
         <v>341</v>
       </c>
       <c r="I105" s="2" t="s">
         <v>342</v>
       </c>
       <c r="K105" s="2" t="s">
-        <v>343</v>
+        <v>126</v>
       </c>
       <c r="L105" s="3" t="s">
         <v>126</v>
@@ -5577,45 +5584,53 @@
       <c r="O105" s="3"/>
       <c r="P105" s="3"/>
     </row>
-    <row r="106" spans="1:16" ht="171" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C106" s="3">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E106" s="3"/>
       <c r="F106" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G106" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="G106" s="2" t="s">
+      <c r="H106" s="2" t="s">
         <v>345</v>
       </c>
+      <c r="I106" s="2" t="s">
+        <v>346</v>
+      </c>
       <c r="K106" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="L106" s="3" t="s">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="M106" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="N106" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="N106" s="3">
+        <v>138</v>
+      </c>
       <c r="O106" s="3"/>
       <c r="P106" s="3"/>
     </row>
-    <row r="107" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:16" ht="171" x14ac:dyDescent="0.2">
       <c r="A107" s="3">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C107" s="3">
         <v>2023</v>
@@ -5625,19 +5640,19 @@
       </c>
       <c r="E107" s="3"/>
       <c r="F107" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K107" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L107" s="3" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="M107" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="N107" s="3"/>
       <c r="O107" s="3"/>
@@ -5645,10 +5660,10 @@
     </row>
     <row r="108" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C108" s="3">
         <v>2023</v>
@@ -5658,32 +5673,30 @@
       </c>
       <c r="E108" s="3"/>
       <c r="F108" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K108" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="L108" s="3" t="s">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="M108" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="N108" s="3">
-        <v>138</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="N108" s="3"/>
       <c r="O108" s="3"/>
       <c r="P108" s="3"/>
     </row>
-    <row r="109" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C109" s="3">
         <v>2023</v>
@@ -5693,13 +5706,13 @@
       </c>
       <c r="E109" s="3"/>
       <c r="F109" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K109" s="2" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="L109" s="3" t="s">
         <v>115</v>
@@ -5713,28 +5726,28 @@
       <c r="O109" s="3"/>
       <c r="P109" s="3"/>
     </row>
-    <row r="110" spans="1:16" ht="171" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C110" s="3">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E110" s="3"/>
       <c r="F110" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="G110" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="K110" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="K110" s="2" t="s">
-        <v>352</v>
       </c>
       <c r="L110" s="3" t="s">
         <v>115</v>
@@ -5748,12 +5761,12 @@
       <c r="O110" s="3"/>
       <c r="P110" s="3"/>
     </row>
-    <row r="111" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:16" ht="171" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C111" s="3">
         <v>2024</v>
@@ -5763,19 +5776,19 @@
       </c>
       <c r="E111" s="3"/>
       <c r="F111" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="K111" s="2" t="s">
-        <v>126</v>
+        <v>356</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="M111" s="3" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="N111" s="3">
         <v>138</v>
@@ -5783,317 +5796,319 @@
       <c r="O111" s="3"/>
       <c r="P111" s="3"/>
     </row>
-    <row r="112" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A112" s="3">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C112" s="3">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E112" s="3"/>
       <c r="F112" s="3" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="H112" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K112" s="2" t="s">
-        <v>362</v>
+        <v>126</v>
       </c>
       <c r="L112" s="3" t="s">
-        <v>22</v>
+        <v>126</v>
       </c>
       <c r="M112" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N112" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="N112" s="3">
+        <v>138</v>
+      </c>
       <c r="O112" s="3"/>
       <c r="P112" s="3"/>
     </row>
-    <row r="113" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>16</v>
+        <v>339</v>
       </c>
       <c r="C113" s="3">
-        <v>1945</v>
+        <v>2025</v>
       </c>
       <c r="D113" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="E113" s="3" t="s">
+      <c r="G113" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="F113" s="3"/>
-      <c r="G113" s="2" t="s">
+      <c r="H113" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="K113" s="2"/>
-      <c r="L113" s="3"/>
-      <c r="M113" s="3"/>
-      <c r="N113" s="3">
-        <v>156</v>
-      </c>
+      <c r="K113" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="L113" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M113" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N113" s="3"/>
       <c r="O113" s="3"/>
       <c r="P113" s="3"/>
     </row>
-    <row r="114" spans="1:16" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="C114" s="3">
-        <v>2007</v>
+        <v>1945</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3" t="s">
-        <v>366</v>
-      </c>
+        <v>367</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="F114" s="3"/>
       <c r="G114" s="2" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="K114" s="2"/>
       <c r="L114" s="3"/>
       <c r="M114" s="3"/>
       <c r="N114" s="3">
-        <v>77</v>
+        <v>156</v>
       </c>
       <c r="O114" s="3"/>
       <c r="P114" s="3"/>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:16" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="C115" s="3">
-        <v>1973</v>
+        <v>2007</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E115" s="3"/>
       <c r="F115" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="K115" s="2"/>
       <c r="L115" s="3"/>
       <c r="M115" s="3"/>
       <c r="N115" s="3">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="O115" s="3"/>
       <c r="P115" s="3"/>
     </row>
-    <row r="116" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C116" s="3">
-        <v>1969</v>
+        <v>1973</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E116" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="F116" s="3"/>
+        <v>85</v>
+      </c>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3" t="s">
+        <v>372</v>
+      </c>
       <c r="G116" s="2" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="K116" s="2"/>
       <c r="L116" s="3"/>
       <c r="M116" s="3"/>
       <c r="N116" s="3">
-        <v>13</v>
-      </c>
-      <c r="O116" s="3">
-        <v>129</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="O116" s="3"/>
       <c r="P116" s="3"/>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="C117" s="3">
-        <v>2006</v>
+        <v>1969</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E117" s="3"/>
-      <c r="F117" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="G117" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="F117" s="3"/>
+      <c r="G117" s="2" t="s">
+        <v>375</v>
+      </c>
       <c r="K117" s="2"/>
       <c r="L117" s="3"/>
       <c r="M117" s="3"/>
       <c r="N117" s="3">
-        <v>75</v>
-      </c>
-      <c r="O117" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="O117" s="3">
+        <v>129</v>
+      </c>
       <c r="P117" s="3"/>
     </row>
-    <row r="118" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C118" s="3">
-        <v>2003</v>
+        <v>2006</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E118" s="3"/>
       <c r="F118" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="G118" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="H118" s="2" t="s">
-        <v>375</v>
-      </c>
+        <v>376</v>
+      </c>
+      <c r="G118" s="2"/>
       <c r="K118" s="2"/>
       <c r="L118" s="3"/>
       <c r="M118" s="3"/>
       <c r="N118" s="3">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="O118" s="3"/>
       <c r="P118" s="3"/>
     </row>
     <row r="119" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A119" s="3">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="C119" s="3">
-        <v>1986</v>
+        <v>2003</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="E119" s="3" t="s">
-        <v>376</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="E119" s="3"/>
       <c r="F119" s="3" t="s">
         <v>377</v>
       </c>
       <c r="G119" s="2" t="s">
         <v>378</v>
+      </c>
+      <c r="H119" s="2" t="s">
+        <v>379</v>
       </c>
       <c r="K119" s="2"/>
       <c r="L119" s="3"/>
       <c r="M119" s="3"/>
       <c r="N119" s="3">
-        <v>144</v>
-      </c>
-      <c r="O119" s="3">
-        <v>146</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="O119" s="3"/>
       <c r="P119" s="3"/>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>271</v>
+        <v>84</v>
       </c>
       <c r="C120" s="3">
-        <v>2011</v>
+        <v>1986</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E120" s="3"/>
+        <v>367</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>380</v>
+      </c>
       <c r="F120" s="3" t="s">
-        <v>325</v>
+        <v>381</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="K120" s="2"/>
       <c r="L120" s="3"/>
       <c r="M120" s="3"/>
       <c r="N120" s="3">
-        <v>104</v>
-      </c>
-      <c r="O120" s="3"/>
+        <v>144</v>
+      </c>
+      <c r="O120" s="3">
+        <v>146</v>
+      </c>
       <c r="P120" s="3"/>
     </row>
-    <row r="121" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>137</v>
+        <v>275</v>
       </c>
       <c r="C121" s="3">
-        <v>1991</v>
+        <v>2011</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E121" s="3" t="s">
-        <v>380</v>
-      </c>
-      <c r="F121" s="3"/>
+        <v>85</v>
+      </c>
+      <c r="E121" s="3"/>
+      <c r="F121" s="3" t="s">
+        <v>329</v>
+      </c>
       <c r="G121" s="2" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="K121" s="2"/>
       <c r="L121" s="3"/>
       <c r="M121" s="3"/>
       <c r="N121" s="3">
-        <v>2</v>
-      </c>
-      <c r="O121" s="3">
-        <v>29</v>
-      </c>
-      <c r="P121" s="3">
-        <v>44</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="O121" s="3"/>
+      <c r="P121" s="3"/>
     </row>
     <row r="122" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>137</v>
@@ -6102,41 +6117,47 @@
         <v>1991</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>363</v>
+        <v>69</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="2" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="K122" s="2"/>
       <c r="L122" s="3"/>
       <c r="M122" s="3"/>
-      <c r="N122" s="3"/>
-      <c r="O122" s="3"/>
-      <c r="P122" s="3"/>
-    </row>
-    <row r="123" spans="1:16" ht="114" x14ac:dyDescent="0.2">
+      <c r="N122" s="3">
+        <v>2</v>
+      </c>
+      <c r="O122" s="3">
+        <v>29</v>
+      </c>
+      <c r="P122" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>271</v>
+        <v>137</v>
       </c>
       <c r="C123" s="3">
-        <v>2010</v>
+        <v>1991</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="2" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="K123" s="2"/>
       <c r="L123" s="3"/>
@@ -6145,25 +6166,25 @@
       <c r="O123" s="3"/>
       <c r="P123" s="3"/>
     </row>
-    <row r="124" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>16</v>
+        <v>275</v>
       </c>
       <c r="C124" s="3">
-        <v>1965</v>
+        <v>2010</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="K124" s="2"/>
       <c r="L124" s="3"/>
@@ -6172,694 +6193,694 @@
       <c r="O124" s="3"/>
       <c r="P124" s="3"/>
     </row>
-    <row r="125" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>271</v>
+        <v>16</v>
       </c>
       <c r="C125" s="3">
-        <v>2020</v>
+        <v>1965</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F125" s="3"/>
       <c r="G125" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="K125" s="2"/>
       <c r="L125" s="3"/>
       <c r="M125" s="3"/>
-      <c r="N125" s="3">
-        <v>89</v>
-      </c>
-      <c r="O125" s="3">
-        <v>105</v>
-      </c>
-      <c r="P125" s="3">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="126" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+      <c r="N125" s="3"/>
+      <c r="O125" s="3"/>
+      <c r="P125" s="3"/>
+    </row>
+    <row r="126" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>16</v>
+        <v>275</v>
       </c>
       <c r="C126" s="3">
-        <v>1929</v>
+        <v>2020</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F126" s="3"/>
       <c r="G126" s="2" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="K126" s="2"/>
       <c r="L126" s="3"/>
       <c r="M126" s="3"/>
-      <c r="N126" s="3"/>
-      <c r="O126" s="3"/>
-      <c r="P126" s="3"/>
-    </row>
-    <row r="127" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+      <c r="N126" s="3">
+        <v>89</v>
+      </c>
+      <c r="O126" s="3">
+        <v>105</v>
+      </c>
+      <c r="P126" s="3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A127" s="3">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>335</v>
+        <v>16</v>
       </c>
       <c r="C127" s="3">
-        <v>2022</v>
+        <v>1929</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>69</v>
+        <v>367</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F127" s="3"/>
       <c r="G127" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="K127" s="2"/>
       <c r="L127" s="3"/>
       <c r="M127" s="3"/>
-      <c r="N127" s="3">
-        <v>108</v>
-      </c>
-      <c r="O127" s="3">
-        <v>109</v>
-      </c>
+      <c r="N127" s="3"/>
+      <c r="O127" s="3"/>
       <c r="P127" s="3"/>
     </row>
-    <row r="128" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A128" s="3">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>84</v>
+        <v>339</v>
       </c>
       <c r="C128" s="3">
-        <v>1983</v>
+        <v>2022</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="F128" s="3"/>
       <c r="G128" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="K128" s="2"/>
       <c r="L128" s="3"/>
       <c r="M128" s="3"/>
       <c r="N128" s="3">
-        <v>23</v>
-      </c>
-      <c r="O128" s="3"/>
+        <v>108</v>
+      </c>
+      <c r="O128" s="3">
+        <v>109</v>
+      </c>
       <c r="P128" s="3"/>
     </row>
-    <row r="129" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A129" s="3">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>137</v>
+        <v>84</v>
       </c>
       <c r="C129" s="3">
-        <v>1997</v>
+        <v>1983</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F129" s="3"/>
       <c r="G129" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="H129" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K129" s="2"/>
       <c r="L129" s="3"/>
       <c r="M129" s="3"/>
       <c r="N129" s="3">
-        <v>55</v>
-      </c>
-      <c r="O129" s="3">
-        <v>50</v>
-      </c>
-      <c r="P129" s="3">
-        <v>58</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="O129" s="3"/>
+      <c r="P129" s="3"/>
     </row>
     <row r="130" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A130" s="3">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="C130" s="3">
-        <v>2007</v>
+        <v>1997</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F130" s="3"/>
       <c r="G130" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>402</v>
       </c>
       <c r="K130" s="2"/>
       <c r="L130" s="3"/>
       <c r="M130" s="3"/>
       <c r="N130" s="3">
-        <v>77</v>
-      </c>
-      <c r="O130" s="3"/>
-      <c r="P130" s="3"/>
+        <v>55</v>
+      </c>
+      <c r="O130" s="3">
+        <v>50</v>
+      </c>
+      <c r="P130" s="3">
+        <v>58</v>
+      </c>
     </row>
     <row r="131" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A131" s="3">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>271</v>
+        <v>120</v>
       </c>
       <c r="C131" s="3">
-        <v>2014</v>
+        <v>2007</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F131" s="3"/>
       <c r="G131" s="2" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K131" s="2"/>
       <c r="L131" s="3"/>
       <c r="M131" s="3"/>
       <c r="N131" s="3">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="O131" s="3"/>
       <c r="P131" s="3"/>
     </row>
-    <row r="132" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:16" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A132" s="3">
+        <v>143</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C132" s="3">
+        <v>2014</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="F132" s="3"/>
+      <c r="G132" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="K132" s="2"/>
+      <c r="L132" s="3"/>
+      <c r="M132" s="3"/>
+      <c r="N132" s="3">
+        <v>93</v>
+      </c>
+      <c r="O132" s="3"/>
+      <c r="P132" s="3"/>
+    </row>
+    <row r="133" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
+      <c r="A133" s="3">
         <v>144</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B133" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C132" s="3">
+      <c r="C133" s="3">
         <v>1986</v>
-      </c>
-      <c r="D132" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E132" s="3"/>
-      <c r="F132" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="G132" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="I132" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="K132" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="L132" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="M132" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="N132" s="3">
-        <v>127</v>
-      </c>
-      <c r="O132" s="3">
-        <v>20</v>
-      </c>
-      <c r="P132" s="3"/>
-    </row>
-    <row r="133" spans="1:16" ht="171" x14ac:dyDescent="0.2">
-      <c r="A133" s="3">
-        <v>145</v>
-      </c>
-      <c r="B133" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C133" s="3">
-        <v>2001</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E133" s="3"/>
       <c r="F133" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="G133" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="G133" s="2" t="s">
+      <c r="I133" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="I133" s="2" t="s">
+      <c r="K133" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="K133" s="2" t="s">
-        <v>406</v>
-      </c>
       <c r="L133" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="M133" s="3" t="s">
         <v>77</v>
       </c>
       <c r="N133" s="3">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="O133" s="3">
-        <v>147</v>
-      </c>
-      <c r="P133" s="3">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="134" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+      <c r="P133" s="3"/>
+    </row>
+    <row r="134" spans="1:16" ht="171" x14ac:dyDescent="0.2">
       <c r="A134" s="3">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C134" s="3">
-        <v>2011</v>
+        <v>2001</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="E134" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="I134" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="K134" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="L134" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="F134" s="3"/>
-      <c r="G134" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="K134" s="2"/>
-      <c r="L134" s="3"/>
-      <c r="M134" s="3"/>
+      <c r="M134" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="N134" s="3">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="O134" s="3">
-        <v>145</v>
-      </c>
-      <c r="P134" s="3"/>
-    </row>
-    <row r="135" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+      <c r="P134" s="3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A135" s="3">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C135" s="3">
-        <v>2001</v>
+        <v>2011</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F135" s="3"/>
       <c r="G135" s="2" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="K135" s="2"/>
       <c r="L135" s="3"/>
       <c r="M135" s="3"/>
       <c r="N135" s="3">
+        <v>127</v>
+      </c>
+      <c r="O135" s="3">
         <v>145</v>
       </c>
-      <c r="O135" s="3"/>
       <c r="P135" s="3"/>
     </row>
-    <row r="136" spans="1:16" ht="114" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A136" s="3">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="C136" s="3">
-        <v>1947</v>
+        <v>2001</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F136" s="3"/>
       <c r="G136" s="2" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="K136" s="2"/>
       <c r="L136" s="3"/>
       <c r="M136" s="3"/>
       <c r="N136" s="3">
-        <v>5</v>
-      </c>
-      <c r="O136" s="3">
-        <v>150</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="O136" s="3"/>
       <c r="P136" s="3"/>
     </row>
     <row r="137" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C137" s="3">
-        <v>1969</v>
+        <v>1947</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E137" s="3"/>
-      <c r="F137" s="3" t="s">
-        <v>417</v>
-      </c>
+        <v>367</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="F137" s="3"/>
       <c r="G137" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="I137" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="J137" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="K137" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L137" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M137" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="K137" s="2"/>
+      <c r="L137" s="3"/>
+      <c r="M137" s="3"/>
       <c r="N137" s="3">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="O137" s="3">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="P137" s="3"/>
     </row>
-    <row r="138" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C138" s="3">
-        <v>1957</v>
+        <v>1969</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E138" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="F138" s="3" t="s">
+      <c r="G138" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="G138" s="2" t="s">
+      <c r="I138" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="K138" s="2"/>
-      <c r="L138" s="3"/>
-      <c r="M138" s="3"/>
+      <c r="J138" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="K138" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L138" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M138" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="N138" s="3">
         <v>148</v>
       </c>
       <c r="O138" s="3">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P138" s="3"/>
     </row>
-    <row r="139" spans="1:16" ht="171" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:16" ht="185.25" x14ac:dyDescent="0.2">
       <c r="A139" s="3">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C139" s="3">
-        <v>1978</v>
+        <v>1957</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="F139" s="3"/>
+        <v>425</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G139" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="J139" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K139" s="2"/>
       <c r="L139" s="3"/>
       <c r="M139" s="3"/>
       <c r="N139" s="3">
-        <v>150</v>
-      </c>
-      <c r="O139" s="3"/>
+        <v>148</v>
+      </c>
+      <c r="O139" s="3">
+        <v>151</v>
+      </c>
       <c r="P139" s="3"/>
     </row>
-    <row r="140" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:16" ht="171" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="C140" s="3">
-        <v>2008</v>
+        <v>1978</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>363</v>
+        <v>69</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F140" s="3"/>
       <c r="G140" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
+      </c>
+      <c r="J140" s="2" t="s">
+        <v>430</v>
       </c>
       <c r="K140" s="2"/>
       <c r="L140" s="3"/>
       <c r="M140" s="3"/>
-      <c r="N140" s="3"/>
+      <c r="N140" s="3">
+        <v>150</v>
+      </c>
       <c r="O140" s="3"/>
       <c r="P140" s="3"/>
     </row>
-    <row r="141" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A141" s="3">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="C141" s="3">
-        <v>1969</v>
+        <v>2008</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F141" s="3"/>
       <c r="G141" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="K141" s="2"/>
       <c r="L141" s="3"/>
       <c r="M141" s="3"/>
-      <c r="N141" s="3">
-        <v>149</v>
-      </c>
-      <c r="O141" s="3">
-        <v>150</v>
-      </c>
-      <c r="P141" s="3">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="142" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
+      <c r="N141" s="3"/>
+      <c r="O141" s="3"/>
+      <c r="P141" s="3"/>
+    </row>
+    <row r="142" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A142" s="3">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="C142" s="3">
-        <v>2003</v>
+        <v>1969</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F142" s="3"/>
       <c r="G142" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="K142" s="2"/>
       <c r="L142" s="3"/>
       <c r="M142" s="3"/>
       <c r="N142" s="3">
-        <v>145</v>
-      </c>
-      <c r="O142" s="3"/>
-      <c r="P142" s="3"/>
-    </row>
-    <row r="143" spans="1:16" ht="171" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+      <c r="O142" s="3">
+        <v>150</v>
+      </c>
+      <c r="P142" s="3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A143" s="3">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C143" s="3">
-        <v>2000</v>
+        <v>2003</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>69</v>
+        <v>367</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="F143" s="3" t="s">
-        <v>434</v>
-      </c>
+        <v>435</v>
+      </c>
+      <c r="F143" s="3"/>
       <c r="G143" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K143" s="2"/>
       <c r="L143" s="3"/>
       <c r="M143" s="3"/>
-      <c r="N143" s="3"/>
+      <c r="N143" s="3">
+        <v>145</v>
+      </c>
       <c r="O143" s="3"/>
       <c r="P143" s="3"/>
     </row>
-    <row r="144" spans="1:16" ht="114" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:16" ht="171" x14ac:dyDescent="0.2">
       <c r="A144" s="3">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>16</v>
+        <v>137</v>
       </c>
       <c r="C144" s="3">
-        <v>1945</v>
+        <v>2000</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>363</v>
+        <v>69</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="F144" s="3"/>
+        <v>437</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>438</v>
+      </c>
       <c r="G144" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="K144" s="2"/>
       <c r="L144" s="3"/>
       <c r="M144" s="3"/>
-      <c r="N144" s="3">
-        <v>119</v>
-      </c>
+      <c r="N144" s="3"/>
       <c r="O144" s="3"/>
       <c r="P144" s="3"/>
     </row>
     <row r="145" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A145" s="3">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>335</v>
+        <v>16</v>
       </c>
       <c r="C145" s="3">
-        <v>2022</v>
+        <v>1945</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F145" s="3"/>
       <c r="G145" s="2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="K145" s="2"/>
       <c r="L145" s="3"/>
       <c r="M145" s="3"/>
-      <c r="N145" s="3"/>
+      <c r="N145" s="3">
+        <v>119</v>
+      </c>
       <c r="O145" s="3"/>
       <c r="P145" s="3"/>
     </row>
-    <row r="146" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:16" ht="114" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>16</v>
+        <v>339</v>
       </c>
       <c r="C146" s="3">
-        <v>1973</v>
+        <v>2022</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F146" s="3"/>
       <c r="G146" s="2" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="K146" s="2"/>
       <c r="L146" s="3"/>
@@ -6868,25 +6889,25 @@
       <c r="O146" s="3"/>
       <c r="P146" s="3"/>
     </row>
-    <row r="147" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:16" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A147" s="3">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>271</v>
+        <v>16</v>
       </c>
       <c r="C147" s="3">
-        <v>2021</v>
+        <v>1973</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F147" s="3"/>
       <c r="G147" s="2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="K147" s="2"/>
       <c r="L147" s="3"/>
@@ -6897,99 +6918,126 @@
     </row>
     <row r="148" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>16</v>
+        <v>275</v>
       </c>
       <c r="C148" s="3">
-        <v>1972</v>
+        <v>2021</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E148" s="3"/>
-      <c r="F148" s="3" t="s">
-        <v>444</v>
-      </c>
+        <v>367</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="F148" s="3"/>
       <c r="G148" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="J148" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="K148" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="L148" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="M148" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="N148" s="3">
-        <v>161</v>
-      </c>
+        <v>447</v>
+      </c>
+      <c r="K148" s="2"/>
+      <c r="L148" s="3"/>
+      <c r="M148" s="3"/>
+      <c r="N148" s="3"/>
       <c r="O148" s="3"/>
       <c r="P148" s="3"/>
     </row>
-    <row r="149" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:16" ht="156.75" x14ac:dyDescent="0.2">
       <c r="A149" s="3">
+        <v>160</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C149" s="3">
+        <v>1972</v>
+      </c>
+      <c r="D149" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E149" s="3"/>
+      <c r="F149" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="J149" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="K149" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="L149" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="M149" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="N149" s="3">
         <v>161</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C149" s="3">
-        <v>1986</v>
-      </c>
-      <c r="D149" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E149" s="3" t="s">
-        <v>447</v>
-      </c>
-      <c r="F149" s="3"/>
-      <c r="G149" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="K149" s="2"/>
-      <c r="L149" s="3"/>
-      <c r="M149" s="3"/>
-      <c r="N149" s="3">
-        <v>160</v>
       </c>
       <c r="O149" s="3"/>
       <c r="P149" s="3"/>
     </row>
-    <row r="150" spans="1:16" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:16" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A150" s="3">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="C150" s="3">
-        <v>1945</v>
+        <v>1986</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E150" s="3"/>
-      <c r="F150" s="3" t="s">
-        <v>24</v>
-      </c>
+      <c r="E150" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="F150" s="3"/>
       <c r="G150" s="2" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="K150" s="2"/>
       <c r="L150" s="3"/>
       <c r="M150" s="3"/>
       <c r="N150" s="3">
-        <v>2</v>
+        <v>160</v>
       </c>
       <c r="O150" s="3"/>
       <c r="P150" s="3"/>
+    </row>
+    <row r="151" spans="1:16" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A151" s="3">
+        <v>162</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C151" s="3">
+        <v>1945</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E151" s="3"/>
+      <c r="F151" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="K151" s="2"/>
+      <c r="L151" s="3"/>
+      <c r="M151" s="3"/>
+      <c r="N151" s="3">
+        <v>2</v>
+      </c>
+      <c r="O151" s="3"/>
+      <c r="P151" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>